<commit_message>
channgement de dossier pour le probleme de drive
</commit_message>
<xml_diff>
--- a/data/raw/lieux_upload.xlsx
+++ b/data/raw/lieux_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,68 +451,68 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HAD MONTROUGE</t>
+          <t>Collège Haut Mesnil</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>FINESS</t>
+          <t>data.education.gouv.fr</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48.81701908628781</v>
+        <v>48.81396906122965</v>
       </c>
       <c r="E2" t="n">
-        <v>2.323909049582313</v>
+        <v>2.307057910317576</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>48.817019086287814, 2.323909049582313</t>
+          <t>48.81396906122965, 2.307057910317576</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HDJ CMP JOAN RIVIERE</t>
+          <t>Collège Maurice Genevoix</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FINESS</t>
+          <t>data.education.gouv.fr</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>48.81678126890864</v>
+        <v>48.81090067352207</v>
       </c>
       <c r="E3" t="n">
-        <v>2.309520981776612</v>
+        <v>2.325197595739604</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>48.81678126890864, 2.309520981776612</t>
+          <t>48.81090067352207, 2.325197595739604</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Aristide Briand</t>
+          <t>Collège Robert Doisneau</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -521,26 +521,26 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>48.81485220472397</v>
+        <v>48.82039933804069</v>
       </c>
       <c r="E4" t="n">
-        <v>2.325926798091101</v>
+        <v>2.316845525624895</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>48.81485220472397, 2.3259267980911007</t>
+          <t>48.820399338040694, 2.3168455256248945</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Buffalo</t>
+          <t>Collège privé Jeanne d'Arc</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -549,26 +549,26 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>48.81117732063301</v>
+        <v>48.8187827836916</v>
       </c>
       <c r="E5" t="n">
-        <v>2.319895452935603</v>
+        <v>2.318516023815689</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>48.811177320633014, 2.3198954529356026</t>
+          <t>48.818782783691596, 2.3185160238156888</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique François Rabelais</t>
+          <t>Ecole secondaire privée Groupe Scolaire Yaguel Yaacov</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -577,26 +577,26 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>48.81921194608093</v>
+        <v>48.81987094409272</v>
       </c>
       <c r="E6" t="n">
-        <v>2.321706931688225</v>
+        <v>2.312216280016048</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>48.81921194608093, 2.321706931688225</t>
+          <t>48.81987094409272, 2.3122162800160475</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Haut-Mesnil</t>
+          <t>Ecole secondaire privée Pardess Hannah</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>COLLEGE</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -605,180 +605,936 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48.81464114560588</v>
+        <v>48.81289063370255</v>
       </c>
       <c r="E7" t="n">
-        <v>2.307565117329271</v>
+        <v>2.319416907837911</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>48.81464114560588, 2.3075651173292706</t>
+          <t>48.81289063370255, 2.3194169078379105</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Marcellin Berthelot</t>
+          <t>HAD MONTROUGE</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>48.81614343118439</v>
+        <v>48.81701908628781</v>
       </c>
       <c r="E8" t="n">
-        <v>2.316528127069811</v>
+        <v>2.323909049582313</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48.816143431184386, 2.3165281270698115</t>
+          <t>48.817019086287814, 2.323909049582313</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Maurice Arnoux</t>
+          <t>HDJ CMP JOAN RIVIERE</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48.82034024428792</v>
+        <v>48.81678126890864</v>
       </c>
       <c r="E9" t="n">
-        <v>2.313280613082784</v>
+        <v>2.309520981776612</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.82034024428792, 2.313280613082784</t>
+          <t>48.81678126890864, 2.309520981776612</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Nicolas Boileau</t>
+          <t>CDS CENTRE MEDICAL MONTROUGE</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre de Santé</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>48.81150373223819</v>
+        <v>48.81326157748526</v>
       </c>
       <c r="E10" t="n">
-        <v>2.317516291018025</v>
+        <v>2.302174343393972</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>48.81150373223819, 2.317516291018025</t>
+          <t>48.81326157748526, 2.302174343393972</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Commissariat de police de Montrouge</t>
+          <t>CDS DENTAIRE AADT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>commissariat</t>
+          <t>Centre de Santé</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>lannuaire.service-public.fr + géocodage BAN</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>48.815784</v>
+        <v>48.81607892733119</v>
       </c>
       <c r="E11" t="n">
-        <v>2.31347</v>
+        <v>2.310158107636889</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>48.815784, 2.31347</t>
+          <t>48.81607892733119, 2.3101581076368887</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mairie de Montrouge</t>
+          <t>CDS DENTAIRE ODONTALIA</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>gare</t>
+          <t>Centre de Santé</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>48.8179643</v>
+        <v>48.81069641347636</v>
       </c>
       <c r="E12" t="n">
-        <v>2.3192501</v>
+        <v>2.31318427643796</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>48.8179643, 2.3192501</t>
+          <t>48.810696413476364, 2.31318427643796</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>CDS HOPSOIN VERDIER</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Centre de Santé</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FINESS</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>48.81611588801121</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.309705474757878</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>48.81611588801121, 2.3097054747578785</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CDS MEDICO DENTAIRE DE MONTROUGE</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Centre de Santé</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FINESS</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>48.81163433501998</v>
+      </c>
+      <c r="E14" t="n">
+        <v>2.3265975234474</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>48.81163433501998, 2.3265975234473997</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CDS MUNICIPAL MONTROUGE</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Centre de Santé</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FINESS</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>48.81717137162057</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2.323960189382609</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>48.81717137162057, 2.3239601893826087</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>CSS DE MONTROUGE</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Centre de santé sexuelle</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FINESS</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>48.81717137162057</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2.323960189382609</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>48.81717137162057, 2.3239601893826087</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>CPTS DE MONTROUGE</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Communautés professionnelles territoriales de santé (CPTS)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FINESS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>48.81691104454355</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2.31850235201646</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>48.816911044543545, 2.3185023520164605</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Ecole primaire Pardess Hannah</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>48.81268773657927</v>
+      </c>
+      <c r="E18" t="n">
+        <v>2.320587970099393</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>48.81268773657927, 2.3205879700993934</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Ecole primaire privée Jeanne d'Arc</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>48.8187827836916</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2.318516023815689</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>48.818782783691596, 2.3185160238156888</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Ecole primaire privée Yaguel Yaacov</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>48.81987094409272</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2.312216280016048</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>48.81987094409272, 2.3122162800160475</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire publique Aristide Briand</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>48.81474745325436</v>
+      </c>
+      <c r="E21" t="n">
+        <v>2.328248729191516</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>48.81474745325436, 2.3282487291915164</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire publique Buffalo</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>48.81150441705952</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2.320162176922167</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>48.81150441705952, 2.3201621769221674</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire publique Nicolas Boileau</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>48.81219093954178</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2.31815958805646</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>48.81219093954178, 2.3181595880564605</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire publique Rabelais</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>48.81892809454184</v>
+      </c>
+      <c r="E24" t="n">
+        <v>2.322403857155729</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>48.81892809454184, 2.322403857155729</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire publique Renaudel</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ECOLE DE NIVEAU ELEMENTAIRE</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>48.81295594973342</v>
+      </c>
+      <c r="E25" t="n">
+        <v>2.308231623428387</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>48.81295594973342, 2.3082316234283873</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Ecole élémentaire d'application Raymond Queneau</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ECOLE ELEMENTAIRE D APPLICATION</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>48.81764028582121</v>
+      </c>
+      <c r="E26" t="n">
+        <v>2.32210598895006</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>48.817640285821206, 2.3221059889500597</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Aristide Briand</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>48.81485220472397</v>
+      </c>
+      <c r="E27" t="n">
+        <v>2.325926798091101</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>48.81485220472397, 2.3259267980911007</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Buffalo</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>48.81117732063301</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2.319895452935603</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>48.811177320633014, 2.3198954529356026</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique François Rabelais</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>48.81921194608093</v>
+      </c>
+      <c r="E29" t="n">
+        <v>2.321706931688225</v>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>48.81921194608093, 2.321706931688225</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Haut-Mesnil</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>48.81464114560588</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2.307565117329271</v>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>48.81464114560588, 2.3075651173292706</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Marcellin Berthelot</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>48.81614343118439</v>
+      </c>
+      <c r="E31" t="n">
+        <v>2.316528127069811</v>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>48.816143431184386, 2.3165281270698115</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Maurice Arnoux</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>48.82034024428792</v>
+      </c>
+      <c r="E32" t="n">
+        <v>2.313280613082784</v>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>48.82034024428792, 2.313280613082784</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Nicolas Boileau</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>48.81150373223819</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2.317516291018025</v>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>48.81150373223819, 2.317516291018025</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Lycée général et technologique Maurice Genevoix</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>LYCEE ENSEIGNT GENERAL ET TECHNOLOGIQUE</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>48.81052663525963</v>
+      </c>
+      <c r="E34" t="n">
+        <v>2.322989622297694</v>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>48.81052663525963, 2.3229896222976945</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Lycée général et technologique privé Jeanne d'Arc</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>LYCEE ENSEIGNT GENERAL ET TECHNOLOGIQUE</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>48.8187827836916</v>
+      </c>
+      <c r="E35" t="n">
+        <v>2.318516023815689</v>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>48.818782783691596, 2.3185160238156888</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Ecole 2D degré professionnel privée - Académie d'Art Dentaire</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>LYCEE PROFESSIONNEL</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>48.81271833109989</v>
+      </c>
+      <c r="E36" t="n">
+        <v>2.322810010821757</v>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>48.81271833109989, 2.322810010821757</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Lycée professionnel Jean Monnet , lycée des métiers de la construction et de la gestion administrative</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>LYCEE PROFESSIONNEL</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>48.81281480460642</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2.305294745262522</v>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>48.81281480460642, 2.3052947452625223</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Commissariat de police de Montrouge</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>commissariat</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>lannuaire.service-public.fr + géocodage BAN</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>48.815784</v>
+      </c>
+      <c r="E38" t="n">
+        <v>2.31347</v>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>48.815784, 2.31347</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mairie de Montrouge</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>gare</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>48.8179643</v>
+      </c>
+      <c r="E39" t="n">
+        <v>2.3192501</v>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>48.8179643, 2.3192501</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>Mairie - Montrouge</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>mairie</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>api-lannuaire.service-public.fr + geocodage BAN</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D40" t="n">
         <v>48.818819</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E40" t="n">
         <v>2.319869</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F40" t="inlineStr">
         <is>
           <t>48.818819, 2.319869</t>
         </is>

</xml_diff>

<commit_message>
bouton interecto(pour le couillon de rayou + voir image pour le couillon de tib)
</commit_message>
<xml_diff>
--- a/data/raw/lieux_upload.xlsx
+++ b/data/raw/lieux_upload.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -731,54 +731,26 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mairie de Montrouge</t>
+          <t>Mairie - Montrouge</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>gare</t>
+          <t>mairie</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>OpenStreetMap</t>
+          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>48.8179643</v>
+        <v>48.818819</v>
       </c>
       <c r="E12" t="n">
-        <v>2.3192501</v>
+        <v>2.319869</v>
       </c>
       <c r="F12" t="inlineStr">
-        <is>
-          <t>48.8179643, 2.3192501</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mairie - Montrouge</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>mairie</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>48.818819</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2.319869</v>
-      </c>
-      <c r="F13" t="inlineStr">
         <is>
           <t>48.818819, 2.319869</t>
         </is>

</xml_diff>

<commit_message>
ajout de la fonctionnalité de recherche d'intersections dans l'index des intersections
</commit_message>
<xml_diff>
--- a/data/raw/lieux_upload.xlsx
+++ b/data/raw/lieux_upload.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HAD MONTROUGE</t>
+          <t>CHI DES ALPES DU SUD</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
+          <t>Centre Hospitalier (C.H.)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,26 +465,26 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48.81701908628781</v>
+        <v>44.55615020845936</v>
       </c>
       <c r="E2" t="n">
-        <v>2.323909049582313</v>
+        <v>6.072879289047154</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>48.817019086287814, 2.323909049582313</t>
+          <t>44.556150208459364, 6.072879289047154</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HDJ CMP JOAN RIVIERE</t>
+          <t>CHI DES ALPES DU SUD SITE DE GAP</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
+          <t>Centre Hospitalier (C.H.)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -493,105 +493,105 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>48.81678126890864</v>
+        <v>44.55639434462401</v>
       </c>
       <c r="E3" t="n">
-        <v>2.309520981776612</v>
+        <v>6.073268072252509</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>48.81678126890864, 2.309520981776612</t>
+          <t>44.55639434462401, 6.073268072252509</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Aristide Briand</t>
+          <t>HJ PSY GEN HELENE CHAIGNEAU GAP</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre Hospitalier (C.H.)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>48.81485220472397</v>
+        <v>44.56544028432427</v>
       </c>
       <c r="E4" t="n">
-        <v>2.325926798091101</v>
+        <v>6.083517547653188</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>48.81485220472397, 2.3259267980911007</t>
+          <t>44.56544028432427, 6.083517547653188</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Buffalo</t>
+          <t>HJ PSY IJ LA DOUCETTE GAP</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre Hospitalier (C.H.)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>48.81117732063301</v>
+        <v>44.56076438993705</v>
       </c>
       <c r="E5" t="n">
-        <v>2.319895452935603</v>
+        <v>6.082004407137266</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>48.811177320633014, 2.3198954529356026</t>
+          <t>44.56076438993705, 6.082004407137266</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique François Rabelais</t>
+          <t>PSY IJ LE CORTO MALTESE GAP</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ECOLE MATERNELLE</t>
+          <t>Centre Hospitalier (C.H.)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>data.education.gouv.fr</t>
+          <t>FINESS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>48.81921194608093</v>
+        <v>44.56532201287292</v>
       </c>
       <c r="E6" t="n">
-        <v>2.321706931688225</v>
+        <v>6.092094563216123</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>48.81921194608093, 2.321706931688225</t>
+          <t>44.56532201287292, 6.092094563216123</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Haut-Mesnil</t>
+          <t>Ecole maternelle Fontreyne</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -605,21 +605,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>48.81464114560588</v>
+        <v>44.5469426518528</v>
       </c>
       <c r="E7" t="n">
-        <v>2.307565117329271</v>
+        <v>6.060859487982519</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>48.81464114560588, 2.3075651173292706</t>
+          <t>44.546942651852795, 6.060859487982519</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Marcellin Berthelot</t>
+          <t>Ecole maternelle Le Rochasson</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -633,21 +633,21 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>48.81614343118439</v>
+        <v>44.56782342061283</v>
       </c>
       <c r="E8" t="n">
-        <v>2.316528127069811</v>
+        <v>6.082189638841484</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>48.816143431184386, 2.3165281270698115</t>
+          <t>44.567823420612825, 6.082189638841484</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ecole maternelle publique Maurice Arnoux</t>
+          <t>Ecole maternelle Paul-Emile Victor</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -661,98 +661,14 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>48.82034024428792</v>
+        <v>44.56961473615492</v>
       </c>
       <c r="E9" t="n">
-        <v>2.313280613082784</v>
+        <v>6.088949619671172</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>48.82034024428792, 2.313280613082784</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Ecole maternelle publique Nicolas Boileau</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>ECOLE MATERNELLE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>data.education.gouv.fr</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>48.81150373223819</v>
-      </c>
-      <c r="E10" t="n">
-        <v>2.317516291018025</v>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>48.81150373223819, 2.317516291018025</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Commissariat de police de Montrouge</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>commissariat</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>lannuaire.service-public.fr + géocodage BAN</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>48.815784</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2.31347</v>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>48.815784, 2.31347</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Mairie - Montrouge</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>mairie</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>48.818819</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2.319869</v>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>48.818819, 2.319869</t>
+          <t>44.56961473615492, 6.088949619671172</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
push pour rayou (upload + IA)
</commit_message>
<xml_diff>
--- a/data/raw/lieux_upload.xlsx
+++ b/data/raw/lieux_upload.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CHI DES ALPES DU SUD</t>
+          <t>HAD MONTROUGE</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Centre Hospitalier (C.H.)</t>
+          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -465,26 +465,26 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>44.55615020845936</v>
+        <v>48.8170190862878</v>
       </c>
       <c r="E2" t="n">
-        <v>6.072879289047154</v>
+        <v>2.323909049582313</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>44.556150208459364, 6.072879289047154</t>
+          <t>48.817019086287814, 2.323909049582313</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CHI DES ALPES DU SUD SITE DE GAP</t>
+          <t>HDJ CMP JOAN RIVIERE</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Centre Hospitalier (C.H.)</t>
+          <t>Centre Hospitalier Spécialisé lutte Maladies Mentales</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -493,105 +493,105 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>44.55639434462401</v>
+        <v>48.81678126890864</v>
       </c>
       <c r="E3" t="n">
-        <v>6.073268072252509</v>
+        <v>2.309520981776612</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>44.55639434462401, 6.073268072252509</t>
+          <t>48.81678126890864, 2.309520981776612</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HJ PSY GEN HELENE CHAIGNEAU GAP</t>
+          <t>Ecole maternelle publique Aristide Briand</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Centre Hospitalier (C.H.)</t>
+          <t>ECOLE MATERNELLE</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FINESS</t>
+          <t>data.education.gouv.fr</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>44.56544028432427</v>
+        <v>48.81485220472397</v>
       </c>
       <c r="E4" t="n">
-        <v>6.083517547653188</v>
+        <v>2.325926798091101</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>44.56544028432427, 6.083517547653188</t>
+          <t>48.81485220472397, 2.3259267980911007</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HJ PSY IJ LA DOUCETTE GAP</t>
+          <t>Ecole maternelle publique Buffalo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Centre Hospitalier (C.H.)</t>
+          <t>ECOLE MATERNELLE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FINESS</t>
+          <t>data.education.gouv.fr</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>44.56076438993705</v>
+        <v>48.81117732063301</v>
       </c>
       <c r="E5" t="n">
-        <v>6.082004407137266</v>
+        <v>2.319895452935603</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>44.56076438993705, 6.082004407137266</t>
+          <t>48.811177320633014, 2.3198954529356026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PSY IJ LE CORTO MALTESE GAP</t>
+          <t>Ecole maternelle publique François Rabelais</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Centre Hospitalier (C.H.)</t>
+          <t>ECOLE MATERNELLE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FINESS</t>
+          <t>data.education.gouv.fr</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>44.56532201287292</v>
+        <v>48.81921194608093</v>
       </c>
       <c r="E6" t="n">
-        <v>6.092094563216123</v>
+        <v>2.321706931688225</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>44.56532201287292, 6.092094563216123</t>
+          <t>48.81921194608093, 2.321706931688225</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ecole maternelle Fontreyne</t>
+          <t>Ecole maternelle publique Haut-Mesnil</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -605,21 +605,21 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>44.5469426518528</v>
+        <v>48.81464114560588</v>
       </c>
       <c r="E7" t="n">
-        <v>6.060859487982519</v>
+        <v>2.307565117329271</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>44.546942651852795, 6.060859487982519</t>
+          <t>48.81464114560588, 2.3075651173292706</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Ecole maternelle Le Rochasson</t>
+          <t>Ecole maternelle publique Marcellin Berthelot</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -633,21 +633,21 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>44.56782342061283</v>
+        <v>48.81614343118439</v>
       </c>
       <c r="E8" t="n">
-        <v>6.082189638841484</v>
+        <v>2.316528127069811</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>44.567823420612825, 6.082189638841484</t>
+          <t>48.816143431184386, 2.3165281270698115</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ecole maternelle Paul-Emile Victor</t>
+          <t>Ecole maternelle publique Maurice Arnoux</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -661,14 +661,126 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>44.56961473615492</v>
+        <v>48.82034024428792</v>
       </c>
       <c r="E9" t="n">
-        <v>6.088949619671172</v>
+        <v>2.313280613082784</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>44.56961473615492, 6.088949619671172</t>
+          <t>48.82034024428792, 2.313280613082784</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ecole maternelle publique Nicolas Boileau</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ECOLE MATERNELLE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>data.education.gouv.fr</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>48.81150373223819</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.317516291018025</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>48.81150373223819, 2.317516291018025</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Commissariat de police de Montrouge</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>commissariat</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>lannuaire.service-public.fr + géocodage BAN</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>48.815784</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2.31347</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>48.815784, 2.31347</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Mairie - Montrouge</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>mairie</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>api-lannuaire.service-public.fr + geocodage BAN</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>48.818819</v>
+      </c>
+      <c r="E12" t="n">
+        <v>2.319869</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>48.818819, 2.319869</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mairie de Montrouge</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>gare</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ajout particulier</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>48.8183751284591</v>
+      </c>
+      <c r="E13" t="n">
+        <v>2.3194283120155</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>48.818420, 2.319451</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ajout colone traveersées osm accident
</commit_message>
<xml_diff>
--- a/data/raw/lieux_upload.xlsx
+++ b/data/raw/lieux_upload.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -465,7 +465,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>48.8170190862878</v>
+        <v>48.81701908628781</v>
       </c>
       <c r="E2" t="n">
         <v>2.323909049582313</v>
@@ -753,34 +753,6 @@
       <c r="F12" t="inlineStr">
         <is>
           <t>48.818819, 2.319869</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Mairie de Montrouge</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>gare</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>ajout particulier</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>48.8183751284591</v>
-      </c>
-      <c r="E13" t="n">
-        <v>2.3194283120155</v>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>48.818420, 2.319451</t>
         </is>
       </c>
     </row>

</xml_diff>